<commit_message>
docs: publish approved DAR-005
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -754,6 +754,56 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>B-04 UTILITY &amp; SERVICE BLOCK – FINAL DESIGN</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Not stated on drawing</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Not stated on drawing</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>B-04 Utility &amp; Service Block</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Architectural Utility &amp; Service Block / Final Design</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Under Project Controller Review</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Correlated</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Physical inspection completed from controlled /mnt/data/drawings.zip. Compass visibly shows W-up, N-right, E-down, S-left; Project Controller certified this orientation as correct. DAR-005 remains under Project Controller Review pending overall approval.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">

</xml_diff>

<commit_message>
docs: publish approved DAR-006
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -826,6 +826,56 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>NORTH ELEVATION (FACING INTERNAL ROAD / RESORT)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Rev. 00</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>25 May 2025</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>B-04 Sustainability &amp; Resource Management Centre (SRMC)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Architectural Elevation</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Approved / Closed</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Correlated</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Physical inspection completed from controlled /mnt/data/drawings.zip. Project Controller certified the compass orientation as correct. DAR-006 approved/closed; no orientation discrepancy recorded.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">

</xml_diff>

<commit_message>
docs: reconcile controlled DDIF DAR mappings
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -898,6 +898,21 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Architectural master plan</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>DAR-007 - Existing controlled DAR</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Existing controlled DAR</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -920,6 +935,21 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Architectural site plan for eco resort</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>DAR-008 - Existing controlled DAR</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Existing controlled DAR</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -942,6 +972,21 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Architectural west elevation</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>DAR-009 - Existing controlled DAR</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Existing controlled DAR</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -964,6 +1009,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Base Master Plan</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>DAR-010 - Approved Base Master Plan</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>APPROVED BASE MASTER PLAN</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>PRIMARY INTERNAL DPR DEVELOPMENT SPATIAL BASELINE</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2788,6 +2853,26 @@
       <c r="D94" t="inlineStr">
         <is>
           <t>.png</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Government Site Plan</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>DAR-093 - Government / Official Site Plan</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>GOVERNMENT / OFFICIAL SITE PLAN</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>OFFICIAL SITE/PLOT REFERENCE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: publish approved DAR-011
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1051,6 +1051,31 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>BUILDING SECTIONS</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>A-407</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>B-04 Sustainability &amp; Resource Management Centre (SRMC)</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>DAR-011 - Approved</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">

</xml_diff>

<commit_message>
Update AST-000012 Figure 4.3-5 and DAR-012
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1098,6 +1098,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Regional Location, Tourism Influence &amp; Strategic Development Context</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>DAR-012 - Approved</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Figure 4.3-5 revised to align with the Approved Base Master Plan / Figure 4.0-2</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">

</xml_diff>

<commit_message>
Approve AST-000016 Existing Site Context and DAR-016
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1206,6 +1206,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>EXISTING SITE CONTEXT</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>DAR-016 - Approved</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Figure 4.15-1 approved as the Existing Site Context drawing; site bounded by common access road on the north and open canal on the west.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">

</xml_diff>

<commit_message>
Approve AST-000017 Site Opportunities and Constraints and DAR-017
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1248,6 +1248,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SITE OPPORTUNITIES &amp; CONSTRAINTS</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>DAR-017 - Approved</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Figure 4.15-2 approved as the Site Opportunities &amp; Constraints drawing; compass corrected to project orientation with north down, south up, east left and west right.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">

</xml_diff>

<commit_message>
Approve AST-000018 Vegetation and Landscape Character and DAR-018
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1290,6 +1290,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>VEGETATION &amp; LANDSCAPE CHARACTER</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>DAR-018 - Approved</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Figure 4.16-1 approved as the Vegetation &amp; Landscape Character drawing; compass corrected to project orientation with north down, south up, east left and west right.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">

</xml_diff>

<commit_message>
Approve AST-000019 Vegetation and Landscape Character and DAR-019
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1332,6 +1332,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>VEGETATION &amp; LANDSCAPE CHARACTER</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>DAR-019 - Approved</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Figure 4.16-1 approved as the Vegetation &amp; Landscape Character drawing; compass corrected to project orientation with north down, south up, east left and west right.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">

</xml_diff>

<commit_message>
Approve AST-000020 Development Suitability Analysis and DAR-020
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1374,6 +1374,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>DEVELOPMENT SUITABILITY ANALYSIS</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>DAR-020 - Approved</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Figure 4.16-2 approved as the Development Suitability Analysis drawing; compass corrected to project orientation with north down, south up, east left and west right.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">

</xml_diff>

<commit_message>
Approve AST-000021 Development Suitability Analysis and DAR-021
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1416,6 +1416,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>DEVELOPMENT SUITABILITY ANALYSIS</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>DAR-021 - Approved</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Figure 4.16-2 approved as the Development Suitability Analysis drawing; compass corrected to project orientation with north down, south up, east left and west right.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">

</xml_diff>

<commit_message>
Approve AST-000022 Landscape Framework and DAR-022
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1458,6 +1458,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LANDSCAPE FRAMEWORK</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>DAR-022 - Approved</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Figure 4.17-1 approved as the Landscape Framework drawing; compass corrected to project orientation with north down, south up, east left and west right.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">

</xml_diff>

<commit_message>
Approve AST-000023 Blue-Green Infrastructure and DAR-023
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1500,6 +1500,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>BLUE-GREEN INFRASTRUCTURE</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>DAR-023 - Approved</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Figure 4.17-2 approved as the Blue-Green Infrastructure drawing; compass corrected to project orientation with north down, south up, east left and west right.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Approve AST-000024 Ecological Network and DAR-024
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1542,6 +1542,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ECOLOGICAL NETWORK</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>DAR-024 - Approved</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Figure 4.18-1 approved as the Ecological Network drawing; compass corrected to project orientation with north down, south up, east left and west right.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">

</xml_diff>

<commit_message>
Approve AST-000025 Climate Responsive Planning and DAR-025
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1584,6 +1584,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>CLIMATE RESPONSIVE PLANNING</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>DAR-025 - Approved</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Figure 4.18-2 approved as the Climate Responsive Planning drawing; compass corrected to project orientation with north down, south up, east left and west right; prevailing NW and secondary N/NE wind directions corrected; solar orientation reconciled; B-04 climate note corrected.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">

</xml_diff>

<commit_message>
Approve AST-000026 Surface Water and Drainage Plan and DAR-026
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1626,6 +1626,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SURFACE WATER &amp; DRAINAGE PLAN</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>DAR-026 - Approved</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Figure 4.19-1 approved as the Surface Water &amp; Drainage Plan drawing; compass corrected to project orientation with north down, south up, east left and west right. Drainage/fall directions and all other substantive drawing content retained unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">

</xml_diff>

<commit_message>
Approve AST-000027 Landscape Master Plan and DAR-027
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1668,6 +1668,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LANDSCAPE MASTER PLAN</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>DAR-027 - Approved</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Figure 4.19-2 approved as the Landscape Master Plan drawing; compass corrected to project orientation with north down, south up, east left and west right. All other substantive drawing content retained unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">

</xml_diff>

<commit_message>
Approve AST-000028 Services and Utilities Plan and DAR-028
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1710,6 +1710,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SERVICES &amp; UTILITIES PLAN</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>DAR-028 - Approved</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Figure 4.20-1 approved as the Services &amp; Utilities Plan drawing; compass corrected to project orientation with north down, south up, east left and west right. All utility network, drainage/flow directions and other substantive drawing content retained unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">

</xml_diff>

<commit_message>
DAR-029 controlled drawing analysis and DDIF update
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1752,6 +1752,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>GROUND FLOOR PLAN (SERVICES &amp; FACILITIES)</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>DAR-029 - Approved</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Figure 4.21-1 approved as the Ground Floor Plan (Services &amp; Facilities) drawing; compass corrected to project orientation with north down, south up, east left and west right. Substantive drawing content retained unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">

</xml_diff>

<commit_message>
DAR-030 controlled drawing analysis and DDIF update
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1794,6 +1794,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>GROUND FLOOR PLAN (SERVICES &amp; FACILITIES)</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>DAR-030 - Approved</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Figure 4.21-1 approved as the Ground Floor Plan (Services &amp; Facilities) drawing; source compass conforms to the controlled project orientation with north down, south up, east left and west right. No drawing correction required. Substantive drawing content retained unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">

</xml_diff>

<commit_message>
DAR-031 controlled drawing analysis and DDIF update
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1836,6 +1836,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>GROUND FLOOR ARCHITECTURAL PLAN</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>DAR-031 - Approved</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Figure 4.22-1 approved as the Ground Floor Architectural Plan drawing; compass corrected only to the controlled project orientation with north down, south up, east left and west right. No full-sheet rotation, mirroring, site-layout relocation, or substantive architectural drawing-content change was performed.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">

</xml_diff>

<commit_message>
DAR-032 controlled drawing analysis and DDIF update
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1878,6 +1878,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>GROUND FLOOR PLAN (SERVICES &amp; FACILITIES)</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>DAR-032 - Approved</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Figure 4.22-2 approved as the Ground Floor Plan (Services &amp; Facilities) drawing; AST-000032 was compared directly with AST-000031 and confirmed as the related services/facilities companion drawing. The controlled correction is compass-only: north down, south up, east left and west right. No building, road, pond, canal, jetty, entrance, parking, plot, label, schedule, dimension, legend, title-block or other substantive drawing content was changed.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">

</xml_diff>

<commit_message>
DAR-033 controlled drawing analysis and DDIF update
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1920,6 +1920,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>GROUND FLOOR PLAN (SERVICES &amp; FACILITIES)</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>DAR-033 - Approved</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Figure 4.22-3 approved as the Ground Floor Plan (Services &amp; Facilities) drawing; AST-000033 was compared directly with AST-000032 and the preceding Figure 4.22 drawing sequence. The controlled correction is compass-only: north down, south up, east left and west right. No building, road, pond, canal, jetty, entrance, parking, plot, label, schedule, dimension, legend, title-block or other substantive drawing content was changed.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">

</xml_diff>

<commit_message>
DAR-034 controlled drawing analysis and DDIF update
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1962,6 +1962,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GROUND FLOOR PLAN (SERVICES &amp; FACILITIES)</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DAR-034 - Approved</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">APPROVED</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figure 4.22-4 approved as the Ground Floor Plan (Services &amp; Facilities) drawing; AST-000034 was compared directly with AST-000033 and the preceding Figure 4.22 drawing sequence. The controlled correction is compass-only: north down, south up, east left and west right. The observed drawing-content difference from AST-000033, including the absence of cottage C-06 in AST-000034, is preserved as source drawing content and was not altered. No building, road, pond, canal, jetty, entrance, parking, plot, label, schedule, dimension, legend, title-block or other substantive drawing content was changed.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">

</xml_diff>

<commit_message>
DAR-038 controlled drawing analysis and DDIF update
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -2070,6 +2070,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SITE SETTING-OUT &amp; DIMENSION PLAN</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>DAR-038 - Approved</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Figure 4.22-5 approved as the Site Setting-Out &amp; Dimension Plan drawing; AST-000038 was compared directly with AST-000034 and the preceding approved Figure 4.22 drawing sequence. The controlled correction is compass-only: north down, south up, east left and west right. The site-setting-out, plot boundaries, coordinates, dimensions, setbacks, levels, access, roads, landscape, water features, buildings, labels, schedules, notes, legend and title-block content were preserved as source drawing content. No substantive drawing-content change was made.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">

</xml_diff>

<commit_message>
DAR-039 controlled drawing analysis and DDIF update
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -2112,6 +2112,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>DIMENSION PLAN</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DAR-039 - Approved</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>AST-000039 approved as the Dimension Plan drawing. AST-000039 was compared directly with AST-000038, which is controlled as the Site Setting-Out &amp; Dimension Plan drawing; the two assets retain their distinct drawing identities and source content. The controlled correction is compass-only: north down, south up, east left and west right. All substantive AST-000039 source drawing content was preserved unchanged, including site geometry, plot boundaries, coordinates, dimensions, setbacks, levels, access, roads, landscape, water features, buildings, labels, schedules, notes, legend and title-block content. No full-sheet rotation, mirroring, relocation, redesign or substantive drawing-content change was made.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">

</xml_diff>

<commit_message>
DAR-040 controlled drawing analysis and DDIF update
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -2154,6 +2154,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>GROUND FLOOR PLAN (SERVICES &amp; FACILITIES)</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DAR-040 - Approved</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>COMPASS ONLY</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">

</xml_diff>

<commit_message>
DAR-041 controlled drawing analysis and DDIF update
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -2196,6 +2196,26 @@
           <t>.png</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>COTTAGE FLOOR PLAN (TYPICAL)</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>DAR-041 - Approved</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>COMPASS ONLY</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">

</xml_diff>

<commit_message>
docs: establish DAR-043 premium couple cottage design basis
</commit_message>
<xml_diff>
--- a/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
+++ b/00_PROJECT_CONTROL/Repository_Database/DDIF-001_Initial_Inventory_Register_v1.1.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master_Drawing_Inventory" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repository_Correlation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drawing_Analysis_Tracker" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facility_Summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revision_History" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Master_Drawing_Inventory" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Repository_Correlation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Drawing_Analysis_Tracker" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Facility_Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Revision_History" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1964,22 +1964,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">GROUND FLOOR PLAN (SERVICES &amp; FACILITIES)</t>
+          <t>GROUND FLOOR PLAN (SERVICES &amp; FACILITIES)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAR-034 - Approved</t>
+          <t>DAR-034 - Approved</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t xml:space="preserve">APPROVED</t>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Figure 4.22-4 approved as the Ground Floor Plan (Services &amp; Facilities) drawing; AST-000034 was compared directly with AST-000033 and the preceding Figure 4.22 drawing sequence. The controlled correction is compass-only: north down, south up, east left and west right. The observed drawing-content difference from AST-000033, including the absence of cottage C-06 in AST-000034, is preserved as source drawing content and was not altered. No building, road, pond, canal, jetty, entrance, parking, plot, label, schedule, dimension, legend, title-block or other substantive drawing content was changed.</t>
+          <t>Figure 4.22-4 approved as the Ground Floor Plan (Services &amp; Facilities) drawing; AST-000034 was compared directly with AST-000033 and the preceding Figure 4.22 drawing sequence. The controlled correction is compass-only: north down, south up, east left and west right. The observed drawing-content difference from AST-000033, including the absence of cottage C-06 in AST-000034, is preserved as source drawing content and was not altered. No building, road, pond, canal, jetty, entrance, parking, plot, label, schedule, dimension, legend, title-block or other substantive drawing content was changed.</t>
         </is>
       </c>
     </row>
@@ -2247,17 +2247,57 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ChatGPT Image Jul 18, 2026, 01_28_20 AM.png</t>
+          <t>AST-000043_PREMIUM_COUPLE_COTTAGE_DESIGN_STUDY_v1.2.png</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>drawings/Current/ChatGPT Image Jul 18, 2026, 01_28_20 AM.png</t>
+          <t>drawings/Current/AST-000043_PREMIUM_COUPLE_COTTAGE_DESIGN_STUDY_v1.2.png</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
           <t>.png</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>PREMIUM COUPLE COTTAGE - ONE-BEDROOM DESIGN STUDY</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>05_Cottage_Type_B</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>PREMIUM COUPLE COTTAGE / DESIGN STUDY</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>APPROVED WORKING BASIS</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>APPROVED - FORMALLY REDESIGNATED UNDER DEC-000004</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>SELECTED FOR HYBRID DPR - 2 KEYS</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>drawings/Current/AST-000043_PREMIUM_COUPLE_COTTAGE_DESIGN_STUDY_v1.2.png</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>AST-000043 formally redesignated from its prior A-004 Typical Eco Cottage source to the approved Premium Couple Cottage design-study basis under DEC-000004. The prior A-004 source PNG is preserved in drawings/Superseded. This v1.2 design study retains the approved West-side entrance, East-side private deck, standard cottage deck basis, one-bedroom king accommodation, couple lounge, premium bathroom with rain shower and vanity, and mini-bar/beverage pantry. AST-041 remains unchanged. AST-000042 remains rejected/duplicate. No new AST, drawing number, or revision has been assigned. Area figures remain preliminary design-study values pending detailed structural and services coordination. Detailed engineering and construction documentation remain deferred.</t>
         </is>
       </c>
     </row>
@@ -3474,7 +3514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3578,6 +3618,33 @@
       <c r="A12" t="inlineStr">
         <is>
           <t>10_Guest_Recreation_Wellness</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>06_Premium_Couple_Cottage</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2 keys</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>New independent one-bedroom Premium Couple Cottage; approved working Hybrid DPR basis under DEC-000004</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>King bedroom; couple lounge; premium bathroom; rain shower; premium vanity; mini-bar/beverage pantry; premium FF&amp;E/lighting; private deck</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>APPROVED WORKING BASIS</t>
         </is>
       </c>
     </row>

</xml_diff>